<commit_message>
NPB自動更新(1軍): 2026-09-10 (steps: all)
</commit_message>
<xml_diff>
--- a/data/プロ野球/2026年/1軍/レギュラーシーズン/games/datamart/2026-09-10.xlsx
+++ b/data/プロ野球/2026年/1軍/レギュラーシーズン/games/datamart/2026-09-10.xlsx
@@ -93133,7 +93133,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2本塁打を放ち、チームの全得点に絡む活躍で勝利に貢献した。</t>
+          <t>2回裏に先制弾、4回裏にもソロを放ち、1試合2本塁打の活躍でチームを牽引。</t>
         </is>
       </c>
     </row>
@@ -93158,7 +93158,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>6回1/3を投げ9奪三振3失点。要所で粘り、試合を支配した。</t>
+          <t>6回1/3を投げ9奪三振3失点の力投。要所で三振を奪い試合を支配した。</t>
         </is>
       </c>
     </row>
@@ -93183,7 +93183,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8回裏に勝ち越しタイムリーを放ち、接戦を制する決定打となった。</t>
+          <t>8回裏にライトへの勝ち越しタイムリーを放ち、接戦を制する決勝打となった。</t>
         </is>
       </c>
     </row>
@@ -93208,7 +93208,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>7回を無失点に抑える好投で、相手打線を完璧に封じ込めた。</t>
+          <t>7回を投げ被安打5無失点の好投。相手打線を完璧に抑え込み試合を作った。</t>
         </is>
       </c>
     </row>
@@ -93233,7 +93233,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>7回1失点の安定した投球で試合を作り、チームの勝利を呼び込んだ。</t>
+          <t>7回1失点6奪三振の安定した投球で試合を作り、チームの勝利に貢献した。</t>
         </is>
       </c>
     </row>
@@ -93248,17 +93248,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ネビン</t>
+          <t>ダルベック</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>西武</t>
+          <t>巨人</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>9回表にダメ押し2ランを放ち、勝利を決定づける猛打賞の活躍。</t>
+          <t>3回裏に勝ち越し2ランホームランを放ち、試合の流れを大きく引き寄せた。</t>
         </is>
       </c>
     </row>

</xml_diff>